<commit_message>
📊 Monthly data update: 2026-07-17
</commit_message>
<xml_diff>
--- a/data/historical_data.xlsx
+++ b/data/historical_data.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Historical Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Deliveries June 2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Summary June 2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Deliveries July 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary July 2026" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -117,6 +119,11 @@
       <color rgb="0064748B"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001A5276"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -200,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -230,6 +237,90 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -382,7 +473,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -508,7 +598,162 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly Deliveries — July 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries July 2026'!B3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="0033A0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries July 2026'!$A$4:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries July 2026'!$B$4:$B$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries July 2026'!C3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="00AEEF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries July 2026'!$A$4:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries July 2026'!$C$4:$C$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Aircraft Delivered</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -824,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1096,6 +1341,96 @@
       </c>
       <c r="AB3" s="8" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C4" s="36" t="n">
+        <v>250</v>
+      </c>
+      <c r="D4" s="36" t="n">
+        <v>324</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>6758</v>
+      </c>
+      <c r="F4" s="36" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G4" s="36" t="n">
+        <v>196</v>
+      </c>
+      <c r="H4" s="36" t="n">
+        <v>33</v>
+      </c>
+      <c r="I4" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="J4" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" s="37" t="n">
+        <v>262</v>
+      </c>
+      <c r="L4" s="37" t="n">
+        <v>815</v>
+      </c>
+      <c r="M4" s="37" t="n">
+        <v>9031</v>
+      </c>
+      <c r="N4" s="37" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="O4" s="37" t="n">
+        <v>193</v>
+      </c>
+      <c r="P4" s="37" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q4" s="37" t="n">
+        <v>21</v>
+      </c>
+      <c r="R4" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="S4" s="38" t="n">
+        <v>214.34</v>
+      </c>
+      <c r="T4" s="38" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="U4" s="38" t="n">
+        <v>254.35</v>
+      </c>
+      <c r="V4" s="38" t="n">
+        <v>176.77</v>
+      </c>
+      <c r="W4" s="38" t="n">
+        <v>192.94</v>
+      </c>
+      <c r="X4" s="38" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="Y4" s="38" t="n">
+        <v>221.3</v>
+      </c>
+      <c r="Z4" s="38" t="n">
+        <v>157.42</v>
+      </c>
+      <c r="AA4" s="35" t="inlineStr">
+        <is>
+          <t>fallback_verified</t>
+        </is>
+      </c>
+      <c r="AB4" s="35" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:AB1"/>
@@ -1496,4 +1831,417 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Monthly Deliveries 2026 YTD — July 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B3" s="41" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="42" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="D3" s="43" t="inlineStr">
+        <is>
+          <t>Combined</t>
+        </is>
+      </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>Boeing Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="n">
+        <v>46</v>
+      </c>
+      <c r="C4" s="45" t="n">
+        <v>19</v>
+      </c>
+      <c r="D4" s="46" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" s="47" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="n">
+        <v>51</v>
+      </c>
+      <c r="C5" s="50" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="51" t="n">
+        <v>86</v>
+      </c>
+      <c r="E5" s="52" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="n">
+        <v>46</v>
+      </c>
+      <c r="C6" s="45" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" s="46" t="n">
+        <v>106</v>
+      </c>
+      <c r="E6" s="53" t="n">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="n">
+        <v>47</v>
+      </c>
+      <c r="C7" s="50" t="n">
+        <v>67</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>114</v>
+      </c>
+      <c r="E7" s="54" t="n">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="45" t="n">
+        <v>81</v>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>141</v>
+      </c>
+      <c r="E8" s="53" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>TOTAL YTD</t>
+        </is>
+      </c>
+      <c r="B11" s="57" t="n">
+        <v>250</v>
+      </c>
+      <c r="C11" s="58" t="n">
+        <v>262</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>512</v>
+      </c>
+      <c r="E11" s="59" t="n">
+        <v>-12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>EuroAir Intel — July 2026 Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="41" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="42" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>Deliveries YTD</t>
+        </is>
+      </c>
+      <c r="B4" s="44" t="n">
+        <v>250</v>
+      </c>
+      <c r="C4" s="45" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>Gross Orders YTD</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="n">
+        <v>324</v>
+      </c>
+      <c r="C5" s="50" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Total Backlog (ac)</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C6" s="45" t="n">
+        <v>9031</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>Backlog Runway (yrs)</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C7" s="50" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>Narrowbody Deliv.</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="n">
+        <v>196</v>
+      </c>
+      <c r="C8" s="45" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>Widebody Deliv.</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="n">
+        <v>45</v>
+      </c>
+      <c r="C9" s="50" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>Stock Price</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>$214.34 USD</t>
+        </is>
+      </c>
+      <c r="C10" s="45" t="inlineStr">
+        <is>
+          <t>€192.94 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>Stock Change Today</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>-1.73%</t>
+        </is>
+      </c>
+      <c r="C11" s="50" t="inlineStr">
+        <is>
+          <t>-1.37%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>52-Week High</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>$254.35</t>
+        </is>
+      </c>
+      <c r="C12" s="45" t="inlineStr">
+        <is>
+          <t>€221.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>52-Week Low</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>$176.77</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>€157.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-07-17</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A1:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
📊 Monthly data update: 2026-09-15
</commit_message>
<xml_diff>
--- a/data/historical_data.xlsx
+++ b/data/historical_data.xlsx
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Historical Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Deliveries June 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary June 2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Deliveries July 2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Summary July 2026" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries June 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary June 2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries July 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary July 2026" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries September 2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary September 2026" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -207,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -375,6 +377,90 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -472,13 +558,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -502,10 +588,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="0033A0"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -529,10 +615,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00AEEF"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -572,8 +658,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -599,14 +685,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -630,10 +715,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="0033A0"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -657,10 +742,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00AEEF"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -700,8 +785,136 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Aircraft Delivered</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly Deliveries — September 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries September 2026'!B3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0033A0"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries September 2026'!$A$4:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries September 2026'!$B$4:$B$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries September 2026'!C3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="00AEEF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries September 2026'!$A$4:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries September 2026'!$C$4:$C$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -727,7 +940,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -742,9 +955,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -754,7 +967,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -769,9 +982,36 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1069,7 +1309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1252,94 +1492,94 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="35" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="36" t="n">
         <v>250</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="36" t="n">
         <v>324</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="36" t="n">
         <v>6758</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="F3" s="36" t="n">
         <v>10.1</v>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="G3" s="36" t="n">
         <v>196</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="36" t="n">
         <v>33</v>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="I3" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="J3" s="36" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="10" t="n">
+      <c r="K3" s="37" t="n">
         <v>262</v>
       </c>
-      <c r="L3" s="10" t="n">
+      <c r="L3" s="37" t="n">
         <v>815</v>
       </c>
-      <c r="M3" s="10" t="n">
+      <c r="M3" s="37" t="n">
         <v>9031</v>
       </c>
-      <c r="N3" s="10" t="n">
+      <c r="N3" s="37" t="n">
         <v>10.4</v>
       </c>
-      <c r="O3" s="10" t="n">
+      <c r="O3" s="37" t="n">
         <v>193</v>
       </c>
-      <c r="P3" s="10" t="n">
+      <c r="P3" s="37" t="n">
         <v>38</v>
       </c>
-      <c r="Q3" s="10" t="n">
+      <c r="Q3" s="37" t="n">
         <v>21</v>
       </c>
-      <c r="R3" s="10" t="n">
+      <c r="R3" s="37" t="n">
         <v>10</v>
       </c>
-      <c r="S3" s="8" t="n">
+      <c r="S3" s="35" t="n">
         <v>222.72</v>
       </c>
-      <c r="T3" s="8" t="n">
+      <c r="T3" s="35" t="n">
         <v>-1.29</v>
       </c>
-      <c r="U3" s="8" t="n">
+      <c r="U3" s="35" t="n">
         <v>254.35</v>
       </c>
-      <c r="V3" s="8" t="n">
+      <c r="V3" s="35" t="n">
         <v>176.77</v>
       </c>
-      <c r="W3" s="8" t="n">
+      <c r="W3" s="35" t="n">
         <v>189.42</v>
       </c>
-      <c r="X3" s="8" t="n">
+      <c r="X3" s="35" t="n">
         <v>-1.31</v>
       </c>
-      <c r="Y3" s="8" t="n">
+      <c r="Y3" s="35" t="n">
         <v>221.3</v>
       </c>
-      <c r="Z3" s="8" t="n">
+      <c r="Z3" s="35" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA3" s="8" t="inlineStr">
+      <c r="AA3" s="35" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB3" s="8" t="inlineStr"/>
+      <c r="AB3" s="35" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="35" t="inlineStr">
@@ -1430,6 +1670,96 @@
         </is>
       </c>
       <c r="AB4" s="35" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>September 2026</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="n">
+        <v>250</v>
+      </c>
+      <c r="D5" s="64" t="n">
+        <v>324</v>
+      </c>
+      <c r="E5" s="64" t="n">
+        <v>6758</v>
+      </c>
+      <c r="F5" s="64" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G5" s="64" t="n">
+        <v>196</v>
+      </c>
+      <c r="H5" s="64" t="n">
+        <v>33</v>
+      </c>
+      <c r="I5" s="64" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="64" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" s="65" t="n">
+        <v>262</v>
+      </c>
+      <c r="L5" s="65" t="n">
+        <v>815</v>
+      </c>
+      <c r="M5" s="65" t="n">
+        <v>9031</v>
+      </c>
+      <c r="N5" s="65" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="O5" s="65" t="n">
+        <v>193</v>
+      </c>
+      <c r="P5" s="65" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="65" t="n">
+        <v>21</v>
+      </c>
+      <c r="R5" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="S5" s="66" t="n">
+        <v>210.27</v>
+      </c>
+      <c r="T5" s="66" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="U5" s="66" t="n">
+        <v>254.35</v>
+      </c>
+      <c r="V5" s="66" t="n">
+        <v>176.77</v>
+      </c>
+      <c r="W5" s="66" t="n">
+        <v>196.04</v>
+      </c>
+      <c r="X5" s="66" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="Y5" s="66" t="n">
+        <v>221.3</v>
+      </c>
+      <c r="Z5" s="66" t="n">
+        <v>157.42</v>
+      </c>
+      <c r="AA5" s="63" t="inlineStr">
+        <is>
+          <t>fallback_verified</t>
+        </is>
+      </c>
+      <c r="AB5" s="63" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1456,7 +1786,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — June 2026</t>
         </is>
@@ -1464,162 +1794,162 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="42" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="43" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="40" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="44" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="45" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="46" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="19" t="n">
+      <c r="E4" s="47" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="48" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="49" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="50" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="51" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="52" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="44" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="45" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="46" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="53" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="49" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="50" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="51" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="54" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="44" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="45" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="46" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="53" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="55" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B10" s="29" t="n">
+      <c r="B10" s="57" t="n">
         <v>250</v>
       </c>
-      <c r="C10" s="30" t="n">
+      <c r="C10" s="58" t="n">
         <v>262</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="40" t="n">
         <v>512</v>
       </c>
-      <c r="E10" s="31" t="n">
+      <c r="E10" s="59" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -1647,7 +1977,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="39" t="inlineStr">
         <is>
           <t>EuroAir Intel — June 2026 Summary</t>
         </is>
@@ -1655,170 +1985,170 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="42" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="44" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="45" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="61" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="49" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="50" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="44" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="45" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="61" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="49" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="50" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="60" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="44" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="45" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="61" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="49" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="50" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="44" t="inlineStr">
         <is>
           <t>$222.72 USD</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>€189.42 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="49" t="inlineStr">
         <is>
           <t>-1.29%</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" s="50" t="inlineStr">
         <is>
           <t>-1.31%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="60" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="61" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="49" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C13" s="50" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="34" t="inlineStr">
+      <c r="A15" s="62" t="inlineStr">
         <is>
           <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-06-19</t>
         </is>
@@ -2244,4 +2574,455 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>Monthly Deliveries 2026 YTD — September 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="68" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B3" s="69" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="70" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="D3" s="71" t="inlineStr">
+        <is>
+          <t>Combined</t>
+        </is>
+      </c>
+      <c r="E3" s="68" t="inlineStr">
+        <is>
+          <t>Boeing Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="72" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B4" s="73" t="n">
+        <v>46</v>
+      </c>
+      <c r="C4" s="74" t="n">
+        <v>19</v>
+      </c>
+      <c r="D4" s="75" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" s="76" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B5" s="77" t="n">
+        <v>51</v>
+      </c>
+      <c r="C5" s="78" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="79" t="n">
+        <v>86</v>
+      </c>
+      <c r="E5" s="80" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="72" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B6" s="73" t="n">
+        <v>46</v>
+      </c>
+      <c r="C6" s="74" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" s="75" t="n">
+        <v>106</v>
+      </c>
+      <c r="E6" s="81" t="n">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="63" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B7" s="77" t="n">
+        <v>47</v>
+      </c>
+      <c r="C7" s="78" t="n">
+        <v>67</v>
+      </c>
+      <c r="D7" s="79" t="n">
+        <v>114</v>
+      </c>
+      <c r="E7" s="82" t="n">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="72" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B8" s="73" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="74" t="n">
+        <v>81</v>
+      </c>
+      <c r="D8" s="75" t="n">
+        <v>141</v>
+      </c>
+      <c r="E8" s="81" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="63" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="63" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="B11" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="72" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="68" t="inlineStr">
+        <is>
+          <t>TOTAL YTD</t>
+        </is>
+      </c>
+      <c r="B13" s="85" t="n">
+        <v>250</v>
+      </c>
+      <c r="C13" s="86" t="n">
+        <v>262</v>
+      </c>
+      <c r="D13" s="68" t="n">
+        <v>512</v>
+      </c>
+      <c r="E13" s="87" t="n">
+        <v>-12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="67" t="inlineStr">
+        <is>
+          <t>EuroAir Intel — September 2026 Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="68" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="69" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="70" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="88" t="inlineStr">
+        <is>
+          <t>Deliveries YTD</t>
+        </is>
+      </c>
+      <c r="B4" s="73" t="n">
+        <v>250</v>
+      </c>
+      <c r="C4" s="74" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="89" t="inlineStr">
+        <is>
+          <t>Gross Orders YTD</t>
+        </is>
+      </c>
+      <c r="B5" s="77" t="n">
+        <v>324</v>
+      </c>
+      <c r="C5" s="78" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="88" t="inlineStr">
+        <is>
+          <t>Total Backlog (ac)</t>
+        </is>
+      </c>
+      <c r="B6" s="73" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C6" s="74" t="n">
+        <v>9031</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="89" t="inlineStr">
+        <is>
+          <t>Backlog Runway (yrs)</t>
+        </is>
+      </c>
+      <c r="B7" s="77" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C7" s="78" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="88" t="inlineStr">
+        <is>
+          <t>Narrowbody Deliv.</t>
+        </is>
+      </c>
+      <c r="B8" s="73" t="n">
+        <v>196</v>
+      </c>
+      <c r="C8" s="74" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="89" t="inlineStr">
+        <is>
+          <t>Widebody Deliv.</t>
+        </is>
+      </c>
+      <c r="B9" s="77" t="n">
+        <v>45</v>
+      </c>
+      <c r="C9" s="78" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="88" t="inlineStr">
+        <is>
+          <t>Stock Price</t>
+        </is>
+      </c>
+      <c r="B10" s="73" t="inlineStr">
+        <is>
+          <t>$210.27 USD</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="inlineStr">
+        <is>
+          <t>€196.04 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="89" t="inlineStr">
+        <is>
+          <t>Stock Change Today</t>
+        </is>
+      </c>
+      <c r="B11" s="77" t="inlineStr">
+        <is>
+          <t>-0.09%</t>
+        </is>
+      </c>
+      <c r="C11" s="78" t="inlineStr">
+        <is>
+          <t>+0.53%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="88" t="inlineStr">
+        <is>
+          <t>52-Week High</t>
+        </is>
+      </c>
+      <c r="B12" s="73" t="inlineStr">
+        <is>
+          <t>$254.35</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>€221.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="89" t="inlineStr">
+        <is>
+          <t>52-Week Low</t>
+        </is>
+      </c>
+      <c r="B13" s="77" t="inlineStr">
+        <is>
+          <t>$176.77</t>
+        </is>
+      </c>
+      <c r="C13" s="78" t="inlineStr">
+        <is>
+          <t>€157.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="90" t="inlineStr">
+        <is>
+          <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-09-15</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A1:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
📊 Monthly data update: 2026-09-16
</commit_message>
<xml_diff>
--- a/data/historical_data.xlsx
+++ b/data/historical_data.xlsx
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -455,6 +455,87 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1492,152 +1573,152 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="72" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="B3" s="35" t="inlineStr">
+      <c r="B3" s="72" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="C3" s="36" t="n">
+      <c r="C3" s="83" t="n">
         <v>250</v>
       </c>
-      <c r="D3" s="36" t="n">
+      <c r="D3" s="83" t="n">
         <v>324</v>
       </c>
-      <c r="E3" s="36" t="n">
+      <c r="E3" s="83" t="n">
         <v>6758</v>
       </c>
-      <c r="F3" s="36" t="n">
+      <c r="F3" s="83" t="n">
         <v>10.1</v>
       </c>
-      <c r="G3" s="36" t="n">
+      <c r="G3" s="83" t="n">
         <v>196</v>
       </c>
-      <c r="H3" s="36" t="n">
+      <c r="H3" s="83" t="n">
         <v>33</v>
       </c>
-      <c r="I3" s="36" t="n">
+      <c r="I3" s="83" t="n">
         <v>12</v>
       </c>
-      <c r="J3" s="36" t="n">
+      <c r="J3" s="83" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="37" t="n">
+      <c r="K3" s="84" t="n">
         <v>262</v>
       </c>
-      <c r="L3" s="37" t="n">
+      <c r="L3" s="84" t="n">
         <v>815</v>
       </c>
-      <c r="M3" s="37" t="n">
+      <c r="M3" s="84" t="n">
         <v>9031</v>
       </c>
-      <c r="N3" s="37" t="n">
+      <c r="N3" s="84" t="n">
         <v>10.4</v>
       </c>
-      <c r="O3" s="37" t="n">
+      <c r="O3" s="84" t="n">
         <v>193</v>
       </c>
-      <c r="P3" s="37" t="n">
+      <c r="P3" s="84" t="n">
         <v>38</v>
       </c>
-      <c r="Q3" s="37" t="n">
+      <c r="Q3" s="84" t="n">
         <v>21</v>
       </c>
-      <c r="R3" s="37" t="n">
+      <c r="R3" s="84" t="n">
         <v>10</v>
       </c>
-      <c r="S3" s="35" t="n">
+      <c r="S3" s="72" t="n">
         <v>222.72</v>
       </c>
-      <c r="T3" s="35" t="n">
+      <c r="T3" s="72" t="n">
         <v>-1.29</v>
       </c>
-      <c r="U3" s="35" t="n">
+      <c r="U3" s="72" t="n">
         <v>254.35</v>
       </c>
-      <c r="V3" s="35" t="n">
+      <c r="V3" s="72" t="n">
         <v>176.77</v>
       </c>
-      <c r="W3" s="35" t="n">
+      <c r="W3" s="72" t="n">
         <v>189.42</v>
       </c>
-      <c r="X3" s="35" t="n">
+      <c r="X3" s="72" t="n">
         <v>-1.31</v>
       </c>
-      <c r="Y3" s="35" t="n">
+      <c r="Y3" s="72" t="n">
         <v>221.3</v>
       </c>
-      <c r="Z3" s="35" t="n">
+      <c r="Z3" s="72" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA3" s="35" t="inlineStr">
+      <c r="AA3" s="72" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB3" s="35" t="inlineStr"/>
+      <c r="AB3" s="72" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="B4" s="35" t="inlineStr">
+      <c r="B4" s="72" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="C4" s="36" t="n">
+      <c r="C4" s="83" t="n">
         <v>250</v>
       </c>
-      <c r="D4" s="36" t="n">
+      <c r="D4" s="83" t="n">
         <v>324</v>
       </c>
-      <c r="E4" s="36" t="n">
+      <c r="E4" s="83" t="n">
         <v>6758</v>
       </c>
-      <c r="F4" s="36" t="n">
+      <c r="F4" s="83" t="n">
         <v>10.1</v>
       </c>
-      <c r="G4" s="36" t="n">
+      <c r="G4" s="83" t="n">
         <v>196</v>
       </c>
-      <c r="H4" s="36" t="n">
+      <c r="H4" s="83" t="n">
         <v>33</v>
       </c>
-      <c r="I4" s="36" t="n">
+      <c r="I4" s="83" t="n">
         <v>12</v>
       </c>
-      <c r="J4" s="36" t="n">
+      <c r="J4" s="83" t="n">
         <v>9</v>
       </c>
-      <c r="K4" s="37" t="n">
+      <c r="K4" s="84" t="n">
         <v>262</v>
       </c>
-      <c r="L4" s="37" t="n">
+      <c r="L4" s="84" t="n">
         <v>815</v>
       </c>
-      <c r="M4" s="37" t="n">
+      <c r="M4" s="84" t="n">
         <v>9031</v>
       </c>
-      <c r="N4" s="37" t="n">
+      <c r="N4" s="84" t="n">
         <v>10.4</v>
       </c>
-      <c r="O4" s="37" t="n">
+      <c r="O4" s="84" t="n">
         <v>193</v>
       </c>
-      <c r="P4" s="37" t="n">
+      <c r="P4" s="84" t="n">
         <v>38</v>
       </c>
-      <c r="Q4" s="37" t="n">
+      <c r="Q4" s="84" t="n">
         <v>21</v>
       </c>
-      <c r="R4" s="37" t="n">
+      <c r="R4" s="84" t="n">
         <v>10</v>
       </c>
       <c r="S4" s="38" t="n">
@@ -1664,102 +1745,102 @@
       <c r="Z4" s="38" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA4" s="35" t="inlineStr">
+      <c r="AA4" s="72" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB4" s="35" t="inlineStr"/>
+      <c r="AB4" s="72" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="91" t="inlineStr">
         <is>
           <t>September 2026</t>
         </is>
       </c>
-      <c r="B5" s="63" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="C5" s="64" t="n">
+      <c r="B5" s="91" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C5" s="91" t="n">
         <v>250</v>
       </c>
-      <c r="D5" s="64" t="n">
+      <c r="D5" s="91" t="n">
         <v>324</v>
       </c>
-      <c r="E5" s="64" t="n">
+      <c r="E5" s="91" t="n">
         <v>6758</v>
       </c>
-      <c r="F5" s="64" t="n">
+      <c r="F5" s="91" t="n">
         <v>10.1</v>
       </c>
-      <c r="G5" s="64" t="n">
+      <c r="G5" s="91" t="n">
         <v>196</v>
       </c>
-      <c r="H5" s="64" t="n">
+      <c r="H5" s="91" t="n">
         <v>33</v>
       </c>
-      <c r="I5" s="64" t="n">
+      <c r="I5" s="91" t="n">
         <v>12</v>
       </c>
-      <c r="J5" s="64" t="n">
+      <c r="J5" s="91" t="n">
         <v>9</v>
       </c>
-      <c r="K5" s="65" t="n">
+      <c r="K5" s="91" t="n">
         <v>262</v>
       </c>
-      <c r="L5" s="65" t="n">
+      <c r="L5" s="91" t="n">
         <v>815</v>
       </c>
-      <c r="M5" s="65" t="n">
+      <c r="M5" s="91" t="n">
         <v>9031</v>
       </c>
-      <c r="N5" s="65" t="n">
+      <c r="N5" s="91" t="n">
         <v>10.4</v>
       </c>
-      <c r="O5" s="65" t="n">
+      <c r="O5" s="91" t="n">
         <v>193</v>
       </c>
-      <c r="P5" s="65" t="n">
+      <c r="P5" s="91" t="n">
         <v>38</v>
       </c>
-      <c r="Q5" s="65" t="n">
+      <c r="Q5" s="91" t="n">
         <v>21</v>
       </c>
-      <c r="R5" s="65" t="n">
+      <c r="R5" s="91" t="n">
         <v>10</v>
       </c>
-      <c r="S5" s="66" t="n">
-        <v>210.27</v>
-      </c>
-      <c r="T5" s="66" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="U5" s="66" t="n">
+      <c r="S5" s="91" t="n">
+        <v>209.69</v>
+      </c>
+      <c r="T5" s="91" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="U5" s="91" t="n">
         <v>254.35</v>
       </c>
-      <c r="V5" s="66" t="n">
+      <c r="V5" s="91" t="n">
         <v>176.77</v>
       </c>
-      <c r="W5" s="66" t="n">
-        <v>196.04</v>
-      </c>
-      <c r="X5" s="66" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="Y5" s="66" t="n">
+      <c r="W5" s="91" t="n">
+        <v>195.6</v>
+      </c>
+      <c r="X5" s="91" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Y5" s="91" t="n">
         <v>221.3</v>
       </c>
-      <c r="Z5" s="66" t="n">
+      <c r="Z5" s="91" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA5" s="63" t="inlineStr">
+      <c r="AA5" s="91" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB5" s="63" t="inlineStr"/>
+      <c r="AB5" s="91" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1786,7 +1867,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — June 2026</t>
         </is>
@@ -1794,162 +1875,162 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="70" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="43" t="inlineStr">
+      <c r="D3" s="71" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="40" t="inlineStr">
+      <c r="E3" s="68" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="44" t="n">
+      <c r="B4" s="73" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="45" t="n">
+      <c r="C4" s="74" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="46" t="n">
+      <c r="D4" s="75" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="47" t="n">
+      <c r="E4" s="76" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="77" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="78" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="51" t="n">
+      <c r="D5" s="79" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="52" t="n">
+      <c r="E5" s="80" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="73" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="74" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="46" t="n">
+      <c r="D6" s="75" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="53" t="n">
+      <c r="E6" s="81" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="77" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="78" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="79" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="54" t="n">
+      <c r="E7" s="82" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="72" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="44" t="n">
+      <c r="B8" s="73" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="74" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="46" t="n">
+      <c r="D8" s="75" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="53" t="n">
+      <c r="E8" s="81" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="55" t="n">
+      <c r="B9" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="56" t="n">
+      <c r="C9" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="51" t="n">
+      <c r="D9" s="79" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="52" t="n">
+      <c r="E9" s="80" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B10" s="57" t="n">
+      <c r="B10" s="85" t="n">
         <v>250</v>
       </c>
-      <c r="C10" s="58" t="n">
+      <c r="C10" s="86" t="n">
         <v>262</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="68" t="n">
         <v>512</v>
       </c>
-      <c r="E10" s="59" t="n">
+      <c r="E10" s="87" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -1977,7 +2058,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>EuroAir Intel — June 2026 Summary</t>
         </is>
@@ -1985,170 +2066,170 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="70" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="88" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="44" t="n">
+      <c r="B4" s="73" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="45" t="n">
+      <c r="C4" s="74" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="89" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="77" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="78" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="88" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="73" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="74" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="89" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="77" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="78" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="88" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="44" t="n">
+      <c r="B8" s="73" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="74" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="89" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="77" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="50" t="n">
+      <c r="C9" s="78" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="88" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="73" t="inlineStr">
         <is>
           <t>$222.72 USD</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C10" s="74" t="inlineStr">
         <is>
           <t>€189.42 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="89" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>-1.29%</t>
         </is>
       </c>
-      <c r="C11" s="50" t="inlineStr">
+      <c r="C11" s="78" t="inlineStr">
         <is>
           <t>-1.31%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="88" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B12" s="73" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
+      <c r="C12" s="74" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="89" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="50" t="inlineStr">
+      <c r="C13" s="78" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr">
+      <c r="A15" s="90" t="inlineStr">
         <is>
           <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-06-19</t>
         </is>
@@ -2180,7 +2261,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — July 2026</t>
         </is>
@@ -2188,181 +2269,181 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="70" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="43" t="inlineStr">
+      <c r="D3" s="71" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="40" t="inlineStr">
+      <c r="E3" s="68" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="35" t="inlineStr">
+      <c r="A4" s="72" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="44" t="n">
+      <c r="B4" s="73" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="45" t="n">
+      <c r="C4" s="74" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="46" t="n">
+      <c r="D4" s="75" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="47" t="n">
+      <c r="E4" s="76" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="48" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="77" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="78" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="51" t="n">
+      <c r="D5" s="79" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="52" t="n">
+      <c r="E5" s="80" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
+      <c r="A6" s="72" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="73" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="74" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="46" t="n">
+      <c r="D6" s="75" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="53" t="n">
+      <c r="E6" s="81" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="48" t="inlineStr">
+      <c r="A7" s="63" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="77" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="78" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="79" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="54" t="n">
+      <c r="E7" s="82" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="35" t="inlineStr">
+      <c r="A8" s="72" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="44" t="n">
+      <c r="B8" s="73" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="74" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="46" t="n">
+      <c r="D8" s="75" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="53" t="n">
+      <c r="E8" s="81" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="63" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="55" t="n">
+      <c r="B9" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="56" t="n">
+      <c r="C9" s="65" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="51" t="n">
+      <c r="D9" s="79" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="52" t="n">
+      <c r="E9" s="80" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="35" t="inlineStr">
+      <c r="A10" s="72" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
+      <c r="B10" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="37" t="n">
+      <c r="C10" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="46" t="n">
+      <c r="D10" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="47" t="n">
+      <c r="E10" s="76" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="40" t="inlineStr">
+      <c r="A11" s="68" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B11" s="57" t="n">
+      <c r="B11" s="85" t="n">
         <v>250</v>
       </c>
-      <c r="C11" s="58" t="n">
+      <c r="C11" s="86" t="n">
         <v>262</v>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="68" t="n">
         <v>512</v>
       </c>
-      <c r="E11" s="59" t="n">
+      <c r="E11" s="87" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -2390,7 +2471,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="67" t="inlineStr">
         <is>
           <t>EuroAir Intel — July 2026 Summary</t>
         </is>
@@ -2398,170 +2479,170 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="69" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="70" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="60" t="inlineStr">
+      <c r="A4" s="88" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="44" t="n">
+      <c r="B4" s="73" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="45" t="n">
+      <c r="C4" s="74" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="61" t="inlineStr">
+      <c r="A5" s="89" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="77" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="50" t="n">
+      <c r="C5" s="78" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="60" t="inlineStr">
+      <c r="A6" s="88" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="73" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="45" t="n">
+      <c r="C6" s="74" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="61" t="inlineStr">
+      <c r="A7" s="89" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="49" t="n">
+      <c r="B7" s="77" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="50" t="n">
+      <c r="C7" s="78" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="60" t="inlineStr">
+      <c r="A8" s="88" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="44" t="n">
+      <c r="B8" s="73" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C8" s="74" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="61" t="inlineStr">
+      <c r="A9" s="89" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="77" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="50" t="n">
+      <c r="C9" s="78" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="60" t="inlineStr">
+      <c r="A10" s="88" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="44" t="inlineStr">
+      <c r="B10" s="73" t="inlineStr">
         <is>
           <t>$214.34 USD</t>
         </is>
       </c>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="C10" s="74" t="inlineStr">
         <is>
           <t>€192.94 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="89" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>-1.73%</t>
         </is>
       </c>
-      <c r="C11" s="50" t="inlineStr">
+      <c r="C11" s="78" t="inlineStr">
         <is>
           <t>-1.37%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="60" t="inlineStr">
+      <c r="A12" s="88" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="44" t="inlineStr">
+      <c r="B12" s="73" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="45" t="inlineStr">
+      <c r="C12" s="74" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="61" t="inlineStr">
+      <c r="A13" s="89" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="49" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="50" t="inlineStr">
+      <c r="C13" s="78" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="62" t="inlineStr">
+      <c r="A15" s="90" t="inlineStr">
         <is>
           <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-07-17</t>
         </is>
@@ -2593,7 +2674,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — September 2026</t>
         </is>
@@ -2601,219 +2682,219 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="71" t="inlineStr">
+      <c r="D3" s="96" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="68" t="inlineStr">
+      <c r="E3" s="93" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="97" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="75" t="n">
+      <c r="D4" s="100" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="76" t="n">
+      <c r="E4" s="101" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="91" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="79" t="n">
+      <c r="D5" s="104" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="80" t="n">
+      <c r="E5" s="105" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="97" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="75" t="n">
+      <c r="D6" s="100" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="81" t="n">
+      <c r="E6" s="106" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="91" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="79" t="n">
+      <c r="D7" s="104" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="82" t="n">
+      <c r="E7" s="107" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="97" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="75" t="n">
+      <c r="D8" s="100" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="81" t="n">
+      <c r="E8" s="106" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="91" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="64" t="n">
+      <c r="B9" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="65" t="n">
+      <c r="C9" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="79" t="n">
+      <c r="D9" s="104" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="80" t="n">
+      <c r="E9" s="105" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="72" t="inlineStr">
+      <c r="A10" s="97" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B10" s="83" t="n">
+      <c r="B10" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="84" t="n">
+      <c r="C10" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="75" t="n">
+      <c r="D10" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="76" t="n">
+      <c r="E10" s="101" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="63" t="inlineStr">
+      <c r="A11" s="91" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="B11" s="64" t="n">
+      <c r="B11" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="65" t="n">
+      <c r="C11" s="109" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="79" t="n">
+      <c r="D11" s="104" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="80" t="n">
+      <c r="E11" s="105" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="72" t="inlineStr">
+      <c r="A12" s="97" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B12" s="83" t="n">
+      <c r="B12" s="110" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="84" t="n">
+      <c r="C12" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="75" t="n">
+      <c r="D12" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="76" t="n">
+      <c r="E12" s="101" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="68" t="inlineStr">
+      <c r="A13" s="93" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B13" s="85" t="n">
+      <c r="B13" s="112" t="n">
         <v>250</v>
       </c>
-      <c r="C13" s="86" t="n">
+      <c r="C13" s="113" t="n">
         <v>262</v>
       </c>
-      <c r="D13" s="68" t="n">
+      <c r="D13" s="93" t="n">
         <v>512</v>
       </c>
-      <c r="E13" s="87" t="n">
+      <c r="E13" s="114" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -2841,7 +2922,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>EuroAir Intel — September 2026 Summary</t>
         </is>
@@ -2849,172 +2930,172 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="88" t="inlineStr">
+      <c r="A4" s="115" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="89" t="inlineStr">
+      <c r="A5" s="116" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="88" t="inlineStr">
+      <c r="A6" s="115" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="89" t="inlineStr">
+      <c r="A7" s="116" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="88" t="inlineStr">
+      <c r="A8" s="115" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="89" t="inlineStr">
+      <c r="A9" s="116" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="77" t="n">
+      <c r="B9" s="102" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="78" t="n">
+      <c r="C9" s="103" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="88" t="inlineStr">
+      <c r="A10" s="115" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
-        <is>
-          <t>$210.27 USD</t>
-        </is>
-      </c>
-      <c r="C10" s="74" t="inlineStr">
-        <is>
-          <t>€196.04 EUR</t>
+      <c r="B10" s="98" t="inlineStr">
+        <is>
+          <t>$209.69 USD</t>
+        </is>
+      </c>
+      <c r="C10" s="99" t="inlineStr">
+        <is>
+          <t>€195.6 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="89" t="inlineStr">
+      <c r="A11" s="116" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="77" t="inlineStr">
-        <is>
-          <t>-0.09%</t>
-        </is>
-      </c>
-      <c r="C11" s="78" t="inlineStr">
-        <is>
-          <t>+0.53%</t>
+      <c r="B11" s="102" t="inlineStr">
+        <is>
+          <t>-0.28%</t>
+        </is>
+      </c>
+      <c r="C11" s="103" t="inlineStr">
+        <is>
+          <t>+0.41%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="88" t="inlineStr">
+      <c r="A12" s="115" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="98" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="74" t="inlineStr">
+      <c r="C12" s="99" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="89" t="inlineStr">
+      <c r="A13" s="116" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="77" t="inlineStr">
+      <c r="B13" s="102" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="78" t="inlineStr">
+      <c r="C13" s="103" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="90" t="inlineStr">
-        <is>
-          <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-09-15</t>
+      <c r="A15" s="117" t="inlineStr">
+        <is>
+          <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-09-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Monthly data update: 2026-10-15
</commit_message>
<xml_diff>
--- a/data/historical_data.xlsx
+++ b/data/historical_data.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary July 2026" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries September 2026" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary September 2026" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries October 2026" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary October 2026" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -209,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -542,6 +544,90 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -894,7 +980,6 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -1020,6 +1105,134 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Monthly Deliveries — October 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries October 2026'!B3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0033A0"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries October 2026'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries October 2026'!$B$4:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Deliveries October 2026'!C3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="00AEEF"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Deliveries October 2026'!$A$4:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Deliveries October 2026'!$C$4:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Aircraft Delivered</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -1075,6 +1288,33 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1390,7 +1630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1573,152 +1813,152 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="72" t="inlineStr">
+      <c r="A3" s="97" t="inlineStr">
         <is>
           <t>June 2026</t>
         </is>
       </c>
-      <c r="B3" s="72" t="inlineStr">
+      <c r="B3" s="97" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="C3" s="83" t="n">
+      <c r="C3" s="110" t="n">
         <v>250</v>
       </c>
-      <c r="D3" s="83" t="n">
+      <c r="D3" s="110" t="n">
         <v>324</v>
       </c>
-      <c r="E3" s="83" t="n">
+      <c r="E3" s="110" t="n">
         <v>6758</v>
       </c>
-      <c r="F3" s="83" t="n">
+      <c r="F3" s="110" t="n">
         <v>10.1</v>
       </c>
-      <c r="G3" s="83" t="n">
+      <c r="G3" s="110" t="n">
         <v>196</v>
       </c>
-      <c r="H3" s="83" t="n">
+      <c r="H3" s="110" t="n">
         <v>33</v>
       </c>
-      <c r="I3" s="83" t="n">
+      <c r="I3" s="110" t="n">
         <v>12</v>
       </c>
-      <c r="J3" s="83" t="n">
+      <c r="J3" s="110" t="n">
         <v>9</v>
       </c>
-      <c r="K3" s="84" t="n">
+      <c r="K3" s="111" t="n">
         <v>262</v>
       </c>
-      <c r="L3" s="84" t="n">
+      <c r="L3" s="111" t="n">
         <v>815</v>
       </c>
-      <c r="M3" s="84" t="n">
+      <c r="M3" s="111" t="n">
         <v>9031</v>
       </c>
-      <c r="N3" s="84" t="n">
+      <c r="N3" s="111" t="n">
         <v>10.4</v>
       </c>
-      <c r="O3" s="84" t="n">
+      <c r="O3" s="111" t="n">
         <v>193</v>
       </c>
-      <c r="P3" s="84" t="n">
+      <c r="P3" s="111" t="n">
         <v>38</v>
       </c>
-      <c r="Q3" s="84" t="n">
+      <c r="Q3" s="111" t="n">
         <v>21</v>
       </c>
-      <c r="R3" s="84" t="n">
+      <c r="R3" s="111" t="n">
         <v>10</v>
       </c>
-      <c r="S3" s="72" t="n">
+      <c r="S3" s="97" t="n">
         <v>222.72</v>
       </c>
-      <c r="T3" s="72" t="n">
+      <c r="T3" s="97" t="n">
         <v>-1.29</v>
       </c>
-      <c r="U3" s="72" t="n">
+      <c r="U3" s="97" t="n">
         <v>254.35</v>
       </c>
-      <c r="V3" s="72" t="n">
+      <c r="V3" s="97" t="n">
         <v>176.77</v>
       </c>
-      <c r="W3" s="72" t="n">
+      <c r="W3" s="97" t="n">
         <v>189.42</v>
       </c>
-      <c r="X3" s="72" t="n">
+      <c r="X3" s="97" t="n">
         <v>-1.31</v>
       </c>
-      <c r="Y3" s="72" t="n">
+      <c r="Y3" s="97" t="n">
         <v>221.3</v>
       </c>
-      <c r="Z3" s="72" t="n">
+      <c r="Z3" s="97" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA3" s="72" t="inlineStr">
+      <c r="AA3" s="97" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB3" s="72" t="inlineStr"/>
+      <c r="AB3" s="97" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="97" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="B4" s="72" t="inlineStr">
+      <c r="B4" s="97" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="C4" s="83" t="n">
+      <c r="C4" s="110" t="n">
         <v>250</v>
       </c>
-      <c r="D4" s="83" t="n">
+      <c r="D4" s="110" t="n">
         <v>324</v>
       </c>
-      <c r="E4" s="83" t="n">
+      <c r="E4" s="110" t="n">
         <v>6758</v>
       </c>
-      <c r="F4" s="83" t="n">
+      <c r="F4" s="110" t="n">
         <v>10.1</v>
       </c>
-      <c r="G4" s="83" t="n">
+      <c r="G4" s="110" t="n">
         <v>196</v>
       </c>
-      <c r="H4" s="83" t="n">
+      <c r="H4" s="110" t="n">
         <v>33</v>
       </c>
-      <c r="I4" s="83" t="n">
+      <c r="I4" s="110" t="n">
         <v>12</v>
       </c>
-      <c r="J4" s="83" t="n">
+      <c r="J4" s="110" t="n">
         <v>9</v>
       </c>
-      <c r="K4" s="84" t="n">
+      <c r="K4" s="111" t="n">
         <v>262</v>
       </c>
-      <c r="L4" s="84" t="n">
+      <c r="L4" s="111" t="n">
         <v>815</v>
       </c>
-      <c r="M4" s="84" t="n">
+      <c r="M4" s="111" t="n">
         <v>9031</v>
       </c>
-      <c r="N4" s="84" t="n">
+      <c r="N4" s="111" t="n">
         <v>10.4</v>
       </c>
-      <c r="O4" s="84" t="n">
+      <c r="O4" s="111" t="n">
         <v>193</v>
       </c>
-      <c r="P4" s="84" t="n">
+      <c r="P4" s="111" t="n">
         <v>38</v>
       </c>
-      <c r="Q4" s="84" t="n">
+      <c r="Q4" s="111" t="n">
         <v>21</v>
       </c>
-      <c r="R4" s="84" t="n">
+      <c r="R4" s="111" t="n">
         <v>10</v>
       </c>
       <c r="S4" s="38" t="n">
@@ -1745,12 +1985,12 @@
       <c r="Z4" s="38" t="n">
         <v>157.42</v>
       </c>
-      <c r="AA4" s="72" t="inlineStr">
+      <c r="AA4" s="97" t="inlineStr">
         <is>
           <t>fallback_verified</t>
         </is>
       </c>
-      <c r="AB4" s="72" t="inlineStr"/>
+      <c r="AB4" s="97" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="91" t="inlineStr">
@@ -1841,6 +2081,96 @@
         </is>
       </c>
       <c r="AB5" s="91" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="118" t="inlineStr">
+        <is>
+          <t>October 2026</t>
+        </is>
+      </c>
+      <c r="B6" s="118" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C6" s="119" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" s="119" t="n">
+        <v>324</v>
+      </c>
+      <c r="E6" s="119" t="n">
+        <v>6758</v>
+      </c>
+      <c r="F6" s="119" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G6" s="119" t="n">
+        <v>196</v>
+      </c>
+      <c r="H6" s="119" t="n">
+        <v>33</v>
+      </c>
+      <c r="I6" s="119" t="n">
+        <v>12</v>
+      </c>
+      <c r="J6" s="119" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" s="120" t="n">
+        <v>262</v>
+      </c>
+      <c r="L6" s="120" t="n">
+        <v>815</v>
+      </c>
+      <c r="M6" s="120" t="n">
+        <v>9031</v>
+      </c>
+      <c r="N6" s="120" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="O6" s="120" t="n">
+        <v>193</v>
+      </c>
+      <c r="P6" s="120" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q6" s="120" t="n">
+        <v>21</v>
+      </c>
+      <c r="R6" s="120" t="n">
+        <v>10</v>
+      </c>
+      <c r="S6" s="121" t="n">
+        <v>184.66</v>
+      </c>
+      <c r="T6" s="121" t="n">
+        <v>-0.98</v>
+      </c>
+      <c r="U6" s="121" t="n">
+        <v>254.35</v>
+      </c>
+      <c r="V6" s="121" t="n">
+        <v>176.77</v>
+      </c>
+      <c r="W6" s="121" t="n">
+        <v>193.62</v>
+      </c>
+      <c r="X6" s="121" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="Y6" s="121" t="n">
+        <v>221.3</v>
+      </c>
+      <c r="Z6" s="121" t="n">
+        <v>157.42</v>
+      </c>
+      <c r="AA6" s="118" t="inlineStr">
+        <is>
+          <t>fallback_verified</t>
+        </is>
+      </c>
+      <c r="AB6" s="118" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1867,7 +2197,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — June 2026</t>
         </is>
@@ -1875,162 +2205,162 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="71" t="inlineStr">
+      <c r="D3" s="96" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="68" t="inlineStr">
+      <c r="E3" s="93" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="97" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="75" t="n">
+      <c r="D4" s="100" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="76" t="n">
+      <c r="E4" s="101" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="91" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="79" t="n">
+      <c r="D5" s="104" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="80" t="n">
+      <c r="E5" s="105" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="97" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="75" t="n">
+      <c r="D6" s="100" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="81" t="n">
+      <c r="E6" s="106" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="91" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="79" t="n">
+      <c r="D7" s="104" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="82" t="n">
+      <c r="E7" s="107" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="97" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="75" t="n">
+      <c r="D8" s="100" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="81" t="n">
+      <c r="E8" s="106" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="91" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="80" t="n">
+      <c r="B9" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="105" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="68" t="inlineStr">
+      <c r="A10" s="93" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B10" s="85" t="n">
+      <c r="B10" s="112" t="n">
         <v>250</v>
       </c>
-      <c r="C10" s="86" t="n">
+      <c r="C10" s="113" t="n">
         <v>262</v>
       </c>
-      <c r="D10" s="68" t="n">
+      <c r="D10" s="93" t="n">
         <v>512</v>
       </c>
-      <c r="E10" s="87" t="n">
+      <c r="E10" s="114" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -2058,7 +2388,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>EuroAir Intel — June 2026 Summary</t>
         </is>
@@ -2066,170 +2396,170 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="88" t="inlineStr">
+      <c r="A4" s="115" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="89" t="inlineStr">
+      <c r="A5" s="116" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="88" t="inlineStr">
+      <c r="A6" s="115" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="89" t="inlineStr">
+      <c r="A7" s="116" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="88" t="inlineStr">
+      <c r="A8" s="115" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="89" t="inlineStr">
+      <c r="A9" s="116" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="77" t="n">
+      <c r="B9" s="102" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="78" t="n">
+      <c r="C9" s="103" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="88" t="inlineStr">
+      <c r="A10" s="115" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="98" t="inlineStr">
         <is>
           <t>$222.72 USD</t>
         </is>
       </c>
-      <c r="C10" s="74" t="inlineStr">
+      <c r="C10" s="99" t="inlineStr">
         <is>
           <t>€189.42 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="89" t="inlineStr">
+      <c r="A11" s="116" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="77" t="inlineStr">
+      <c r="B11" s="102" t="inlineStr">
         <is>
           <t>-1.29%</t>
         </is>
       </c>
-      <c r="C11" s="78" t="inlineStr">
+      <c r="C11" s="103" t="inlineStr">
         <is>
           <t>-1.31%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="88" t="inlineStr">
+      <c r="A12" s="115" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="98" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="74" t="inlineStr">
+      <c r="C12" s="99" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="89" t="inlineStr">
+      <c r="A13" s="116" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="77" t="inlineStr">
+      <c r="B13" s="102" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="78" t="inlineStr">
+      <c r="C13" s="103" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="90" t="inlineStr">
+      <c r="A15" s="117" t="inlineStr">
         <is>
           <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-06-19</t>
         </is>
@@ -2261,7 +2591,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>Monthly Deliveries 2026 YTD — July 2026</t>
         </is>
@@ -2269,181 +2599,181 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
-      <c r="D3" s="71" t="inlineStr">
+      <c r="D3" s="96" t="inlineStr">
         <is>
           <t>Combined</t>
         </is>
       </c>
-      <c r="E3" s="68" t="inlineStr">
+      <c r="E3" s="93" t="inlineStr">
         <is>
           <t>Boeing Lead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="72" t="inlineStr">
+      <c r="A4" s="97" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="75" t="n">
+      <c r="D4" s="100" t="n">
         <v>65</v>
       </c>
-      <c r="E4" s="76" t="n">
+      <c r="E4" s="101" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="63" t="inlineStr">
+      <c r="A5" s="91" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>51</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>35</v>
       </c>
-      <c r="D5" s="79" t="n">
+      <c r="D5" s="104" t="n">
         <v>86</v>
       </c>
-      <c r="E5" s="80" t="n">
+      <c r="E5" s="105" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="72" t="inlineStr">
+      <c r="A6" s="97" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>46</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="75" t="n">
+      <c r="D6" s="100" t="n">
         <v>106</v>
       </c>
-      <c r="E6" s="81" t="n">
+      <c r="E6" s="106" t="n">
         <v>-14</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="63" t="inlineStr">
+      <c r="A7" s="91" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>47</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>67</v>
       </c>
-      <c r="D7" s="79" t="n">
+      <c r="D7" s="104" t="n">
         <v>114</v>
       </c>
-      <c r="E7" s="82" t="n">
+      <c r="E7" s="107" t="n">
         <v>-20</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="72" t="inlineStr">
+      <c r="A8" s="97" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>60</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>81</v>
       </c>
-      <c r="D8" s="75" t="n">
+      <c r="D8" s="100" t="n">
         <v>141</v>
       </c>
-      <c r="E8" s="81" t="n">
+      <c r="E8" s="106" t="n">
         <v>-21</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="91" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="80" t="n">
+      <c r="B9" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="105" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="72" t="inlineStr">
+      <c r="A10" s="97" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B10" s="83" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="84" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="76" t="n">
+      <c r="B10" s="110" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="101" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="68" t="inlineStr">
+      <c r="A11" s="93" t="inlineStr">
         <is>
           <t>TOTAL YTD</t>
         </is>
       </c>
-      <c r="B11" s="85" t="n">
+      <c r="B11" s="112" t="n">
         <v>250</v>
       </c>
-      <c r="C11" s="86" t="n">
+      <c r="C11" s="113" t="n">
         <v>262</v>
       </c>
-      <c r="D11" s="68" t="n">
+      <c r="D11" s="93" t="n">
         <v>512</v>
       </c>
-      <c r="E11" s="87" t="n">
+      <c r="E11" s="114" t="n">
         <v>-12</v>
       </c>
     </row>
@@ -2471,7 +2801,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="67" t="inlineStr">
+      <c r="A1" s="92" t="inlineStr">
         <is>
           <t>EuroAir Intel — July 2026 Summary</t>
         </is>
@@ -2479,170 +2809,170 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="68" t="inlineStr">
+      <c r="A3" s="93" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="69" t="inlineStr">
+      <c r="B3" s="94" t="inlineStr">
         <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="C3" s="70" t="inlineStr">
+      <c r="C3" s="95" t="inlineStr">
         <is>
           <t>Airbus</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="88" t="inlineStr">
+      <c r="A4" s="115" t="inlineStr">
         <is>
           <t>Deliveries YTD</t>
         </is>
       </c>
-      <c r="B4" s="73" t="n">
+      <c r="B4" s="98" t="n">
         <v>250</v>
       </c>
-      <c r="C4" s="74" t="n">
+      <c r="C4" s="99" t="n">
         <v>262</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="89" t="inlineStr">
+      <c r="A5" s="116" t="inlineStr">
         <is>
           <t>Gross Orders YTD</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n">
+      <c r="B5" s="102" t="n">
         <v>324</v>
       </c>
-      <c r="C5" s="78" t="n">
+      <c r="C5" s="103" t="n">
         <v>815</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="88" t="inlineStr">
+      <c r="A6" s="115" t="inlineStr">
         <is>
           <t>Total Backlog (ac)</t>
         </is>
       </c>
-      <c r="B6" s="73" t="n">
+      <c r="B6" s="98" t="n">
         <v>6758</v>
       </c>
-      <c r="C6" s="74" t="n">
+      <c r="C6" s="99" t="n">
         <v>9031</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="89" t="inlineStr">
+      <c r="A7" s="116" t="inlineStr">
         <is>
           <t>Backlog Runway (yrs)</t>
         </is>
       </c>
-      <c r="B7" s="77" t="n">
+      <c r="B7" s="102" t="n">
         <v>10.1</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="103" t="n">
         <v>10.4</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="88" t="inlineStr">
+      <c r="A8" s="115" t="inlineStr">
         <is>
           <t>Narrowbody Deliv.</t>
         </is>
       </c>
-      <c r="B8" s="73" t="n">
+      <c r="B8" s="98" t="n">
         <v>196</v>
       </c>
-      <c r="C8" s="74" t="n">
+      <c r="C8" s="99" t="n">
         <v>193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="89" t="inlineStr">
+      <c r="A9" s="116" t="inlineStr">
         <is>
           <t>Widebody Deliv.</t>
         </is>
       </c>
-      <c r="B9" s="77" t="n">
+      <c r="B9" s="102" t="n">
         <v>45</v>
       </c>
-      <c r="C9" s="78" t="n">
+      <c r="C9" s="103" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="88" t="inlineStr">
+      <c r="A10" s="115" t="inlineStr">
         <is>
           <t>Stock Price</t>
         </is>
       </c>
-      <c r="B10" s="73" t="inlineStr">
+      <c r="B10" s="98" t="inlineStr">
         <is>
           <t>$214.34 USD</t>
         </is>
       </c>
-      <c r="C10" s="74" t="inlineStr">
+      <c r="C10" s="99" t="inlineStr">
         <is>
           <t>€192.94 EUR</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="89" t="inlineStr">
+      <c r="A11" s="116" t="inlineStr">
         <is>
           <t>Stock Change Today</t>
         </is>
       </c>
-      <c r="B11" s="77" t="inlineStr">
+      <c r="B11" s="102" t="inlineStr">
         <is>
           <t>-1.73%</t>
         </is>
       </c>
-      <c r="C11" s="78" t="inlineStr">
+      <c r="C11" s="103" t="inlineStr">
         <is>
           <t>-1.37%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="88" t="inlineStr">
+      <c r="A12" s="115" t="inlineStr">
         <is>
           <t>52-Week High</t>
         </is>
       </c>
-      <c r="B12" s="73" t="inlineStr">
+      <c r="B12" s="98" t="inlineStr">
         <is>
           <t>$254.35</t>
         </is>
       </c>
-      <c r="C12" s="74" t="inlineStr">
+      <c r="C12" s="99" t="inlineStr">
         <is>
           <t>€221.3</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="89" t="inlineStr">
+      <c r="A13" s="116" t="inlineStr">
         <is>
           <t>52-Week Low</t>
         </is>
       </c>
-      <c r="B13" s="77" t="inlineStr">
+      <c r="B13" s="102" t="inlineStr">
         <is>
           <t>$176.77</t>
         </is>
       </c>
-      <c r="C13" s="78" t="inlineStr">
+      <c r="C13" s="103" t="inlineStr">
         <is>
           <t>€157.42</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="90" t="inlineStr">
+      <c r="A15" s="117" t="inlineStr">
         <is>
           <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-07-17</t>
         </is>
@@ -3106,4 +3436,474 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="122" t="inlineStr">
+        <is>
+          <t>Monthly Deliveries 2026 YTD — October 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="123" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B3" s="124" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="125" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="D3" s="126" t="inlineStr">
+        <is>
+          <t>Combined</t>
+        </is>
+      </c>
+      <c r="E3" s="123" t="inlineStr">
+        <is>
+          <t>Boeing Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="118" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="B4" s="127" t="n">
+        <v>46</v>
+      </c>
+      <c r="C4" s="128" t="n">
+        <v>19</v>
+      </c>
+      <c r="D4" s="129" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" s="130" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="131" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="B5" s="132" t="n">
+        <v>51</v>
+      </c>
+      <c r="C5" s="133" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="134" t="n">
+        <v>86</v>
+      </c>
+      <c r="E5" s="135" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="118" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="B6" s="127" t="n">
+        <v>46</v>
+      </c>
+      <c r="C6" s="128" t="n">
+        <v>60</v>
+      </c>
+      <c r="D6" s="129" t="n">
+        <v>106</v>
+      </c>
+      <c r="E6" s="136" t="n">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="131" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="B7" s="132" t="n">
+        <v>47</v>
+      </c>
+      <c r="C7" s="133" t="n">
+        <v>67</v>
+      </c>
+      <c r="D7" s="134" t="n">
+        <v>114</v>
+      </c>
+      <c r="E7" s="137" t="n">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="118" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="B8" s="127" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="128" t="n">
+        <v>81</v>
+      </c>
+      <c r="D8" s="129" t="n">
+        <v>141</v>
+      </c>
+      <c r="E8" s="136" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="131" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B9" s="138" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="118" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="B10" s="119" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="129" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="131" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="B11" s="138" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="118" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B12" s="119" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="129" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="131" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B13" s="138" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="123" t="inlineStr">
+        <is>
+          <t>TOTAL YTD</t>
+        </is>
+      </c>
+      <c r="B14" s="140" t="n">
+        <v>250</v>
+      </c>
+      <c r="C14" s="141" t="n">
+        <v>262</v>
+      </c>
+      <c r="D14" s="123" t="n">
+        <v>512</v>
+      </c>
+      <c r="E14" s="142" t="n">
+        <v>-12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="122" t="inlineStr">
+        <is>
+          <t>EuroAir Intel — October 2026 Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="123" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="124" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C3" s="125" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="143" t="inlineStr">
+        <is>
+          <t>Deliveries YTD</t>
+        </is>
+      </c>
+      <c r="B4" s="127" t="n">
+        <v>250</v>
+      </c>
+      <c r="C4" s="128" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="144" t="inlineStr">
+        <is>
+          <t>Gross Orders YTD</t>
+        </is>
+      </c>
+      <c r="B5" s="132" t="n">
+        <v>324</v>
+      </c>
+      <c r="C5" s="133" t="n">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="143" t="inlineStr">
+        <is>
+          <t>Total Backlog (ac)</t>
+        </is>
+      </c>
+      <c r="B6" s="127" t="n">
+        <v>6758</v>
+      </c>
+      <c r="C6" s="128" t="n">
+        <v>9031</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="144" t="inlineStr">
+        <is>
+          <t>Backlog Runway (yrs)</t>
+        </is>
+      </c>
+      <c r="B7" s="132" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C7" s="133" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="143" t="inlineStr">
+        <is>
+          <t>Narrowbody Deliv.</t>
+        </is>
+      </c>
+      <c r="B8" s="127" t="n">
+        <v>196</v>
+      </c>
+      <c r="C8" s="128" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="144" t="inlineStr">
+        <is>
+          <t>Widebody Deliv.</t>
+        </is>
+      </c>
+      <c r="B9" s="132" t="n">
+        <v>45</v>
+      </c>
+      <c r="C9" s="133" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="143" t="inlineStr">
+        <is>
+          <t>Stock Price</t>
+        </is>
+      </c>
+      <c r="B10" s="127" t="inlineStr">
+        <is>
+          <t>$184.66 USD</t>
+        </is>
+      </c>
+      <c r="C10" s="128" t="inlineStr">
+        <is>
+          <t>€193.62 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="144" t="inlineStr">
+        <is>
+          <t>Stock Change Today</t>
+        </is>
+      </c>
+      <c r="B11" s="132" t="inlineStr">
+        <is>
+          <t>-0.98%</t>
+        </is>
+      </c>
+      <c r="C11" s="133" t="inlineStr">
+        <is>
+          <t>+1.79%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="143" t="inlineStr">
+        <is>
+          <t>52-Week High</t>
+        </is>
+      </c>
+      <c r="B12" s="127" t="inlineStr">
+        <is>
+          <t>$254.35</t>
+        </is>
+      </c>
+      <c r="C12" s="128" t="inlineStr">
+        <is>
+          <t>€221.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="144" t="inlineStr">
+        <is>
+          <t>52-Week Low</t>
+        </is>
+      </c>
+      <c r="B13" s="132" t="inlineStr">
+        <is>
+          <t>$176.77</t>
+        </is>
+      </c>
+      <c r="C13" s="133" t="inlineStr">
+        <is>
+          <t>€157.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="145" t="inlineStr">
+        <is>
+          <t>Source: Boeing.com · Airbus.com · Yahoo Finance · Generated 2026-10-15</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A1:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>